<commit_message>
Generate v2026.2 pop file; Add documentation file
</commit_message>
<xml_diff>
--- a/LHJ Data/outputs/final/Data-Dictionary.xlsx
+++ b/LHJ Data/outputs/final/Data-Dictionary.xlsx
@@ -1,26 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\FusionData\Population Task Force\LHJ Data\outputs\final\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5A3C7A0-5434-424E-B8D6-0B70801E7C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C77CBE40-41A6-4E35-89B3-D44C788FBA53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6570" yWindow="4320" windowWidth="23130" windowHeight="12150" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3975" yWindow="2130" windowWidth="32745" windowHeight="17190" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Vintage 2026.2" sheetId="1" r:id="rId1"/>
+    <sheet name="Vintage 2026.1" sheetId="4" r:id="rId2"/>
+    <sheet name="Vintage 2025.2" sheetId="2" r:id="rId3"/>
+    <sheet name="Vintage 2025.1" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="39">
   <si>
     <t>Column</t>
   </si>
@@ -31,18 +34,12 @@
     <t>county_lhj</t>
   </si>
   <si>
-    <t>58 California Counties (Alameda, Alpine, etc), 3 city jurisdictions (Berkeley, Long Beach, Pasadena), Alameda HD, and Los Angeles HD</t>
-  </si>
-  <si>
     <t>year</t>
   </si>
   <si>
     <t>sex</t>
   </si>
   <si>
-    <t>Sex at birth</t>
-  </si>
-  <si>
     <t>age</t>
   </si>
   <si>
@@ -79,16 +76,70 @@
     <t>Annual; Ranges from 2000 to 2030</t>
   </si>
   <si>
-    <t>LHJ Population dataset last updated February 9, 2026</t>
-  </si>
-  <si>
     <t>DOF E6 2020-2025 (released February 2026), DOF E6 2010-2019 (released December 2021), and DOF E6 2000-2010 (released December 2011)</t>
   </si>
   <si>
-    <t xml:space="preserve">California Department of Public Health, Population Data Work Group. (Published February 9, 2026). Local Health Jurisdiction Population Estimates by Age by Race and Ethnicity by Sex [Data set]. https://data.chhs.ca.gov/dataset/cdph-california-population-estimates-by-age-race_ethnicity-sex-at-local-health-jurisdiction-level </t>
-  </si>
-  <si>
     <t>July 1st (mid-year) Population values; 2000-2025 are estimates; 2026-2030 are projections</t>
+  </si>
+  <si>
+    <t>county_indicator</t>
+  </si>
+  <si>
+    <t>lhj_indicator</t>
+  </si>
+  <si>
+    <t>1 if California county; 0 otherwise (Berkeley, Long Beach, Pasadena, Alameda HD, Los Angeles HD)</t>
+  </si>
+  <si>
+    <t>1 if Local Health Jurisdiction; 0 otherwise (Alameda, Los Angeles)</t>
+  </si>
+  <si>
+    <t>58 California Counties (Alameda, Alpine, etc), 3 city jurisdictions (Berkeley, Long Beach, Pasadena), Alameda HD (Health Department), and Los Angeles HD</t>
+  </si>
+  <si>
+    <t>Annual; Ranges from 2000 to 2024</t>
+  </si>
+  <si>
+    <t>DOF E6 2020-2024 (released December 2024), DOF E6 2010-2019 (released December 2021), and DOF E6 2000-2010 (released December 2011)</t>
+  </si>
+  <si>
+    <t>July (mid-year) Population estimates</t>
+  </si>
+  <si>
+    <t>July (mid-year) population estimates</t>
+  </si>
+  <si>
+    <t>PopDaWG LHJ Age-Race-Sex Population File - Vintage 2025.2 (released October 21, 2025)</t>
+  </si>
+  <si>
+    <t>Sex at birth (Female, Male)</t>
+  </si>
+  <si>
+    <t>California Department of Public Health, Population Data Work Group. (Published October 21, 2025). Local Health Jurisdiction Age-Race-Sex Population File - Vintage 2025.2 [Data set]. https://data.chhs.ca.gov/dataset/cdph-california-population-estimates-by-age-race_ethnicity-sex-at-local-health-jurisdiction-level</t>
+  </si>
+  <si>
+    <t>DOF P3 Vintage 2025 (released 2025.04.25)</t>
+  </si>
+  <si>
+    <t>California Department of Public Health, Population Data Work Group. (Published May 21, 2025). Local Health Jurisdiction Age-Race-Sex Population File - Vintage 2025.1 [Data set]. https://data.chhs.ca.gov/dataset/cdph-california-population-estimates-by-age-race_ethnicity-sex-at-local-health-jurisdiction-level</t>
+  </si>
+  <si>
+    <t>PopDaWG LHJ Age-Race-Sex Population File - Vintage 2025.1 (released May 21, 2025)</t>
+  </si>
+  <si>
+    <t>PopDaWG LHJ Age-Race-Sex Population File - Vintage 2026.2 (released April 8, 2026)</t>
+  </si>
+  <si>
+    <t>DOF P3 Vintage 2026 (released 2026.03.13)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">California Department of Public Health, Population Data Work Group. (Published April 8, 2026). Local Health Jurisdiction Age-Race-Sex Population File - Vintage 2026.2 [Data set]. https://data.chhs.ca.gov/dataset/cdph-california-population-estimates-by-age-race_ethnicity-sex-at-local-health-jurisdiction-level </t>
+  </si>
+  <si>
+    <t>PopDaWG LHJ Age-Race-Sex Population File - Vintage 2026.1 (released February 13, 2026)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">California Department of Public Health, Population Data Work Group. (Published February 13, 2026). Local Health Jurisdiction Age-Race-Sex Population File - Vintage 2026.1 [Data set]. https://data.chhs.ca.gov/dataset/cdph-california-population-estimates-by-age-race_ethnicity-sex-at-local-health-jurisdiction-level </t>
   </si>
 </sst>
 </file>
@@ -168,10 +219,40 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:B7" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table3" displayName="Table3" ref="A1:B9" totalsRowShown="0">
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Column"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F637D74A-CC46-4D49-84C7-BCDF55FB6998}" name="Table32" displayName="Table32" ref="A1:B9" totalsRowShown="0">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{8475263D-C5D5-4D86-A751-543C9F5FA48E}" name="Column"/>
+    <tableColumn id="4" xr3:uid="{0D6068AA-8F11-4471-964E-8350A6110D79}" name="Description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{B0D2C5D5-780A-43D4-AE72-A52EF3D90BFB}" name="Table35" displayName="Table35" ref="A1:B7" totalsRowShown="0">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{51546DD4-2CD4-4380-8FD7-7A744355EA2E}" name="Column"/>
+    <tableColumn id="4" xr3:uid="{82324907-2124-4CD9-9A83-0D5500D3D4C6}" name="Description"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{A66C87F8-73D7-4041-9B0F-ACDE4F8493F5}" name="Table36" displayName="Table36" ref="A1:B7" totalsRowShown="0">
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{E4DA7C98-4204-4C14-8F62-1346100653F6}" name="Column"/>
+    <tableColumn id="4" xr3:uid="{923F4597-93B4-4A25-B7C3-0C657E08101E}" name="Description"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -456,6 +537,278 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="200.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>36</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <headerFooter>
+    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Confidential - Low</oddFooter>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E5C08A49-A4B8-4746-9041-2BF513683200}">
+  <dimension ref="A1:B20"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="200.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B16" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B19" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B20" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4EFACC0F-C273-4F0F-930B-A69DF788117F}">
   <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -476,102 +829,216 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>3</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B9" s="3" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B10" s="3" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B11" s="3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B12" s="3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B13" s="3" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B14" s="3" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B15" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B17" s="3" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
-  <headerFooter>
-    <oddFooter>&amp;C_x000D_&amp;1#&amp;"Calibri"&amp;10&amp;K000000 Confidential - Low</oddFooter>
-  </headerFooter>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{397B2B10-497C-43D5-8FCB-6415107E52F9}">
+  <dimension ref="A1:B18"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.7109375" customWidth="1"/>
+    <col min="2" max="2" width="200.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B9" s="3" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B10" s="3" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B11" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B12" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B13" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B14" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="B15" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B17" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B18" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>